<commit_message>
Add Ovalux competitor context
</commit_message>
<xml_diff>
--- a/reports/bozarc_keyword_research.xlsx
+++ b/reports/bozarc_keyword_research.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R77dc574617cc474a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Review" sheetId="2" r:id="Rcf032b2f5ae04f1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recommended Keywords" sheetId="3" r:id="Rcd70d39af58f4add"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carports" sheetId="4" r:id="R52fae9beae2240c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vehicle Carports" sheetId="5" r:id="R0c214dd1e6f0430a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Terras Covers" sheetId="6" r:id="Rd5ddeec68374442c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Terras Options" sheetId="7" r:id="Ra3eeb3480e0048fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Serres Tuinkamers" sheetId="8" r:id="R660a22917e1a46a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B2B Overkappingen" sheetId="9" r:id="Re333969333f840b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geo Variants" sheetId="10" r:id="Rc6cbc33e6a494692"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand" sheetId="11" r:id="R05096e6313924317"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Unclustered" sheetId="12" r:id="R3be408bcdfd54293"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Negatives" sheetId="13" r:id="R658aaf1a686f4117"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference Seeds" sheetId="14" r:id="R8d4cabfb8c734fd1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Google Autosuggest" sheetId="15" r:id="R37472b4c8dd64d4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Autosuggest R2" sheetId="16" r:id="R4a747e299bc84063"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Autosuggest R3" sheetId="17" r:id="R8d5633d7e2ca45f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="18" r:id="R2aae53afd6414bc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R253a5d3a1b2e43ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Review" sheetId="2" r:id="Rc30b917a44024a66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recommended Keywords" sheetId="3" r:id="Rf76e2d7eb16a49c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carports" sheetId="4" r:id="R871fd277b7fc4741"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vehicle Carports" sheetId="5" r:id="Ra5314b7d615e4495"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Terras Covers" sheetId="6" r:id="Rfcefaecbb4a04879"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Terras Options" sheetId="7" r:id="R7f2c15533d524483"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Serres Tuinkamers" sheetId="8" r:id="R8df952eaddd14278"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B2B Overkappingen" sheetId="9" r:id="R8bbc36e0b7794060"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geo Variants" sheetId="10" r:id="R7979990959a2444b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand" sheetId="11" r:id="Re996ff9ce7b44ee8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Unclustered" sheetId="12" r:id="R1a7e169ac2f3465b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Negatives" sheetId="13" r:id="R08fd48ce8bfa479d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference Seeds" sheetId="14" r:id="R8c63a819f9684e9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Google Autosuggest" sheetId="15" r:id="R02815e6cf3bf4077"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Autosuggest R2" sheetId="16" r:id="R1bbc0c56ba5e4a49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Autosuggest R3" sheetId="17" r:id="R9a92494f8a154efc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="18" r:id="R6b6733e042c942cd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -301,8 +301,8 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="NegativesTbl" displayName="NegativesTbl" ref="A4:D31" headerRowCount="1">
-  <x:autoFilter ref="A4:D31"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="NegativesTbl" displayName="NegativesTbl" ref="A4:D32" headerRowCount="1">
+  <x:autoFilter ref="A4:D32"/>
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Negative Keyword"/>
     <x:tableColumn id="2" name="Level (Campaign/Ad Group)"/>
@@ -375,8 +375,8 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="SourcesTbl" displayName="SourcesTbl" ref="A4:D13" headerRowCount="1">
-  <x:autoFilter ref="A4:D13"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="SourcesTbl" displayName="SourcesTbl" ref="A4:D14" headerRowCount="1">
+  <x:autoFilter ref="A4:D14"/>
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Source"/>
     <x:tableColumn id="2" name="Title"/>
@@ -1247,7 +1247,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcba28c0d3c449ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9e886bff1cd4e7f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1845,7 +1845,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc19fd0da771f4dcc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8db9a337543e4688"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2547,7 +2547,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39b1a27927bc4a6d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8704c47f5714641"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2928,13 +2928,13 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="29" t="str">
-        <x:v>groningen</x:v>
+        <x:v>ovalux</x:v>
       </x:c>
       <x:c r="B28" s="30" t="str">
         <x:v>Campaign</x:v>
       </x:c>
       <x:c r="C28" s="30" t="str">
-        <x:v>Wrong-country/wrong-region geo for Belgian-first campaign</x:v>
+        <x:v>Verified Wallonia competitor/entity intent</x:v>
       </x:c>
       <x:c r="D28" s="10" t="str">
         <x:v>All non-brand acquisition</x:v>
@@ -2942,7 +2942,7 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="29" t="str">
-        <x:v>rotterdam</x:v>
+        <x:v>groningen</x:v>
       </x:c>
       <x:c r="B29" s="30" t="str">
         <x:v>Campaign</x:v>
@@ -2956,29 +2956,43 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="29" t="str">
-        <x:v>schoonmaken</x:v>
+        <x:v>rotterdam</x:v>
       </x:c>
       <x:c r="B30" s="30" t="str">
         <x:v>Campaign</x:v>
       </x:c>
       <x:c r="C30" s="30" t="str">
+        <x:v>Wrong-country/wrong-region geo for Belgian-first campaign</x:v>
+      </x:c>
+      <x:c r="D30" s="10" t="str">
+        <x:v>All non-brand acquisition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="29" t="str">
+        <x:v>schoonmaken</x:v>
+      </x:c>
+      <x:c r="B31" s="30" t="str">
+        <x:v>Campaign</x:v>
+      </x:c>
+      <x:c r="C31" s="30" t="str">
         <x:v>Maintenance/cleaning service not supported by reviewed offer</x:v>
       </x:c>
-      <x:c r="D30" s="10" t="str">
+      <x:c r="D31" s="10" t="str">
         <x:v>B2B overkappingen</x:v>
       </x:c>
     </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="31" t="str">
+    <x:row r="32">
+      <x:c r="A32" s="31" t="str">
         <x:v>verwijderen</x:v>
       </x:c>
-      <x:c r="B31" s="32" t="str">
+      <x:c r="B32" s="32" t="str">
         <x:v>Campaign</x:v>
       </x:c>
-      <x:c r="C31" s="32" t="str">
+      <x:c r="C32" s="32" t="str">
         <x:v>Removal service not supported by reviewed offer</x:v>
       </x:c>
-      <x:c r="D31" s="15" t="str">
+      <x:c r="D32" s="15" t="str">
         <x:v>B2B overkappingen</x:v>
       </x:c>
     </x:row>
@@ -2989,7 +3003,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14036dd4de5b4ee1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30188c9d2f9a455f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3347,7 +3361,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R973476868b7045e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9576d99647e4d22"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6500,7 +6514,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4500dfcba4294aa3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7be977c4e1cd4a9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9492,7 +9506,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R850f65370f2145db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R333e25e7fb214675"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11909,7 +11923,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a9904c34dd24ea1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R987ddbfbfd614302"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12052,16 +12066,16 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="29" t="str">
-        <x:v>Autosuggest</x:v>
+        <x:v>Competitor website</x:v>
       </x:c>
       <x:c r="B11" s="30" t="str">
-        <x:v>Google Search Bar UI round 1</x:v>
+        <x:v>Ovalux</x:v>
       </x:c>
       <x:c r="C11" s="30" t="str">
-        <x:v>https://www.google.com/?hl=nl&amp;gl=be&amp;pws=0</x:v>
+        <x:v>https://ovalux.com/</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
-        <x:v>Core product + location seeds collected 2026-06-22 in Dutch/Belgium UI.</x:v>
+        <x:v>Verified Wallonia/Belgium competitor context: aluminium carports and pergolas, including carports for voiture/camping-car, custom quote flow, Florenville/province du Luxembourg contact context.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -12069,26 +12083,40 @@
         <x:v>Autosuggest</x:v>
       </x:c>
       <x:c r="B12" s="30" t="str">
-        <x:v>Google Search Bar UI round 2</x:v>
+        <x:v>Google Search Bar UI round 1</x:v>
       </x:c>
       <x:c r="C12" s="30" t="str">
         <x:v>https://www.google.com/?hl=nl&amp;gl=be&amp;pws=0</x:v>
       </x:c>
       <x:c r="D12" s="10" t="str">
+        <x:v>Core product + location seeds collected 2026-06-22 in Dutch/Belgium UI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="29" t="str">
+        <x:v>Autosuggest</x:v>
+      </x:c>
+      <x:c r="B13" s="30" t="str">
+        <x:v>Google Search Bar UI round 2</x:v>
+      </x:c>
+      <x:c r="C13" s="30" t="str">
+        <x:v>https://www.google.com/?hl=nl&amp;gl=be&amp;pws=0</x:v>
+      </x:c>
+      <x:c r="D13" s="10" t="str">
         <x:v>Modifier and funnel-intent seeds collected 2026-06-22 in Dutch/Belgium UI.</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="31" t="str">
+    <x:row r="14">
+      <x:c r="A14" s="31" t="str">
         <x:v>Autosuggest</x:v>
       </x:c>
-      <x:c r="B13" s="32" t="str">
+      <x:c r="B14" s="32" t="str">
         <x:v>Google Search Bar UI round 3</x:v>
       </x:c>
-      <x:c r="C13" s="32" t="str">
+      <x:c r="C14" s="32" t="str">
         <x:v>https://www.google.com/?hl=nl&amp;gl=be&amp;pws=0</x:v>
       </x:c>
-      <x:c r="D13" s="15" t="str">
+      <x:c r="D14" s="15" t="str">
         <x:v>Validation-gap seeds for offerte/plaatsing intent, B2B buyer wording, geo/showroom risk, and low-fit exclusions.</x:v>
       </x:c>
     </x:row>
@@ -12099,7 +12127,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89b85745030246b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b3c86dcf83e49cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12346,7 +12374,7 @@
         <x:v>DIY, cheap, secondhand, competitor/store and unsupported solar terms</x:v>
       </x:c>
       <x:c r="C14" s="32" t="str">
-        <x:v>terrasoverkapping goedkoop; carport bouwpakket; carport tweedehands; hubo; zonnepanelen</x:v>
+        <x:v>terrasoverkapping goedkoop; carport bouwpakket; carport tweedehands; hubo; gumax; ovalux; zonnepanelen</x:v>
       </x:c>
       <x:c r="D14" s="32" t="str">
         <x:v>These can spend budget on low-fit or unsupported searches unless client explicitly wants them.</x:v>
@@ -12368,7 +12396,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9feb5cdff6304b77"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92ab15780ba0495a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18192,7 +18220,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R260ea87338c642b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41f8d4a7f6134410"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19466,7 +19494,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bb80961a78e4c8d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22e70fc1cdb2461a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20012,7 +20040,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a20cd5cd8c74756"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96f5dec5314b4a8b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21468,7 +21496,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68c94bbc83404331"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8034186b5880453b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21910,7 +21938,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f43345ef1664360"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5213936012f408b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22508,7 +22536,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd020fd5fdafa4787"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bf7ba8ca92c4afe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23184,7 +23212,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbce217fa7274277"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a2c6e6d94db4b46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>